<commit_message>
New Layers with new weights
</commit_message>
<xml_diff>
--- a/Automated_Pipeline/CUSTOM/REPORTS/Indicator_Weights_Summary.xlsx
+++ b/Automated_Pipeline/CUSTOM/REPORTS/Indicator_Weights_Summary.xlsx
@@ -2287,7 +2287,7 @@
         <v>0.0865166382238169</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0333829666170333</v>
+        <v>0.0494100494100494</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
         <v>0.2117831842315003</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0438469561530438</v>
+        <v>0.1209441209441209</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         <v>0.2291557696861398</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2017937982062018</v>
+        <v>0.1312681312681312</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -2395,7 +2395,7 @@
         <v>0.2499095519088195</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1838568161431838</v>
+        <v>0.2647492647492647</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
         <v>0.2973717066747122</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3044336955663044</v>
+        <v>0.1703541703541703</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -2467,7 +2467,7 @@
         <v>0.2142246244199923</v>
       </c>
       <c r="E12" t="n">
-        <v>0.2326857673142327</v>
+        <v>0.2632742632742633</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3867,11 +3867,11 @@
         <v>0.1793107796856119</v>
       </c>
       <c r="E52" t="n">
-        <v>0.1787675082372672</v>
+        <v>0.117996</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>kendall</t>
+          <t>custom</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3903,11 +3903,11 @@
         <v>0.09927208999672819</v>
       </c>
       <c r="E53" t="n">
-        <v>0.0989713178278309</v>
+        <v>0.06526</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>kendall</t>
+          <t>custom</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3939,11 +3939,11 @@
         <v>0.1732225952812849</v>
       </c>
       <c r="E54" t="n">
-        <v>0.1726977696662857</v>
+        <v>0.114041</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>kendall</t>
+          <t>custom</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3975,11 +3975,11 @@
         <v>0.1726001793585464</v>
       </c>
       <c r="E55" t="n">
-        <v>0.1720772395242037</v>
+        <v>0.248517</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>kendall</t>
+          <t>custom</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4011,11 +4011,11 @@
         <v>0.1902249072695776</v>
       </c>
       <c r="E56" t="n">
-        <v>0.1896485684623695</v>
+        <v>0.125247</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>kendall</t>
+          <t>custom</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4047,11 +4047,11 @@
         <v>0.0924605433273403</v>
       </c>
       <c r="E57" t="n">
-        <v>0.09218040861722281</v>
+        <v>0.265656</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>kendall</t>
+          <t>custom</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -4083,11 +4083,11 @@
         <v>0.0959478882479386</v>
       </c>
       <c r="E58" t="n">
-        <v>0.09565718766482</v>
+        <v>0.06328300000000001</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>kendall</t>
+          <t>custom</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -5156,10 +5156,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.3469387755102041</v>
+        <v>0.2959183673469387</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1349206349206349</v>
+        <v>0.1283185840707964</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -5184,10 +5184,10 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.183673469387755</v>
+        <v>0.1326530612244897</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0714285714285714</v>
+        <v>0.0575221238938053</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -5212,10 +5212,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.4693877551020407</v>
+        <v>0.4387755102040816</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1825396825396825</v>
+        <v>0.1902654867256637</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -5240,10 +5240,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.3571428571428571</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1269841269841269</v>
+        <v>0.1548672566371681</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -5268,10 +5268,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.4489795918367346</v>
+        <v>0.3979591836734694</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.1725663716814159</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -5296,10 +5296,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.2448979591836734</v>
+        <v>0.2346938775510203</v>
       </c>
       <c r="E15" t="n">
-        <v>0.09523809523809521</v>
+        <v>0.1017699115044247</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -5324,10 +5324,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.2244897959183673</v>
+        <v>0.2346938775510203</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0873015873015873</v>
+        <v>0.1017699115044247</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -5352,10 +5352,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2142857142857142</v>
       </c>
       <c r="E17" t="n">
-        <v>0.1269841269841269</v>
+        <v>0.09292035398230079</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -5380,10 +5380,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.2342857142857143</v>
+        <v>0.2254945054945055</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1647095179233622</v>
+        <v>0.1609159347553325</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -5408,10 +5408,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.149010989010989</v>
+        <v>0.1481318681318681</v>
       </c>
       <c r="E19" t="n">
-        <v>0.1047589616810877</v>
+        <v>0.1057089084065244</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -5436,10 +5436,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.1551648351648351</v>
+        <v>0.1648351648351648</v>
       </c>
       <c r="E20" t="n">
-        <v>0.1090852904820766</v>
+        <v>0.1176286072772898</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -5464,10 +5464,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.2615384615384616</v>
+        <v>0.2536263736263737</v>
       </c>
       <c r="E21" t="n">
-        <v>0.1838689740420272</v>
+        <v>0.18099121706399</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -5492,10 +5492,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.272967032967033</v>
+        <v>0.2457142857142857</v>
       </c>
       <c r="E22" t="n">
-        <v>0.1919035846724351</v>
+        <v>0.17534504391468</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -5520,10 +5520,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.06285714285714281</v>
+        <v>0.069010989010989</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0441903584672435</v>
+        <v>0.0492471769134253</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -5548,10 +5548,10 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.1305494505494505</v>
+        <v>0.1437362637362637</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0917799752781211</v>
+        <v>0.1025721455457967</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -5576,10 +5576,10 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.156043956043956</v>
+        <v>0.1507692307692307</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1097033374536464</v>
+        <v>0.1075909661229611</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Updates to the layers
</commit_message>
<xml_diff>
--- a/Automated_Pipeline/CUSTOM/REPORTS/Indicator_Weights_Summary.xlsx
+++ b/Automated_Pipeline/CUSTOM/REPORTS/Indicator_Weights_Summary.xlsx
@@ -2084,7 +2084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3428,14 +3428,14 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Faith in elections</t>
+          <t>Demographic Factor</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.1554352806509307</v>
+        <v>0.1310980037857101</v>
       </c>
       <c r="E40" t="n">
-        <v>0.0549619450380549</v>
+        <v>0</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -3464,14 +3464,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Faith in politics</t>
+          <t>Faith in elections</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.1724147150653528</v>
+        <v>0.1591490072633531</v>
       </c>
       <c r="E41" t="n">
-        <v>0.0427479572520427</v>
+        <v>0.0549619450380549</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -3500,14 +3500,14 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ISF effect on quality of life: worsened life somewhat + alot</t>
+          <t>Faith in politics</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.2708911286792593</v>
+        <v>0.165237380242456</v>
       </c>
       <c r="E42" t="n">
-        <v>0.0396949603050396</v>
+        <v>0.0427479572520427</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -3536,14 +3536,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LAF effect on quality of life: worsened life somewhat + alot</t>
+          <t>ISF effect on quality of life: worsened life somewhat + alot</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.2495979667014238</v>
+        <v>0.2598686477891816</v>
       </c>
       <c r="E43" t="n">
-        <v>0.0473279526720473</v>
+        <v>0.0396949603050396</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -3572,14 +3572,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Municipal authorities effect on quality of life: worsened life somewhat + alot</t>
+          <t>LAF effect on quality of life: worsened life somewhat + alot</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.1652535914908379</v>
+        <v>0.2432688551783794</v>
       </c>
       <c r="E44" t="n">
-        <v>0.0587789412210587</v>
+        <v>0.0473279526720473</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -3608,14 +3608,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Municipal council entrenchment</t>
+          <t>Municipal authorities effect on quality of life: worsened life somewhat + alot</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.1231567687088015</v>
+        <v>0.1715002110059001</v>
       </c>
       <c r="E45" t="n">
-        <v>0.2267177732822267</v>
+        <v>0.0587789412210587</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -3644,14 +3644,14 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Municipal elections turnout</t>
+          <t>Municipal council entrenchment</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.1464563770543368</v>
+        <v>0.1136877556707401</v>
       </c>
       <c r="E46" t="n">
-        <v>0.0519079480920519</v>
+        <v>0.2267177732822267</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -3680,14 +3680,14 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">State Citizen Incidents </t>
+          <t>Municipal elections turnout</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.1013540249718007</v>
+        <v>0.1451036849467801</v>
       </c>
       <c r="E47" t="n">
-        <v>0.0358779641220358</v>
+        <v>0.0519079480920519</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -3716,14 +3716,14 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Trust in LAF</t>
+          <t xml:space="preserve">State Citizen Incidents </t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.1042995161796692</v>
+        <v>0.1034531739412614</v>
       </c>
       <c r="E48" t="n">
-        <v>0.0366409633590366</v>
+        <v>0.0358779641220358</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -3752,14 +3752,14 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Trust in Parliament</t>
+          <t>Trust in LAF</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.2205286247443602</v>
+        <v>0.1035566077800814</v>
       </c>
       <c r="E49" t="n">
-        <v>0.07786292213707779</v>
+        <v>0.0366409633590366</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -3788,14 +3788,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Trust in security forces</t>
+          <t>Trust in Parliament</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.2203380747115999</v>
+        <v>0.210369020033815</v>
       </c>
       <c r="E50" t="n">
-        <v>0.2473277526722473</v>
+        <v>0.07786292213707779</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -3824,14 +3824,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Trust in the court system</t>
+          <t>Trust in security forces</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.2264588684632804</v>
+        <v>0.2163576846840651</v>
       </c>
       <c r="E51" t="n">
-        <v>0.0801529198470801</v>
+        <v>0.2473277526722473</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -3851,23 +3851,23 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Gender Based Vulnerabilities</t>
+          <t>Political Vulnerability</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Fear of movement or travel (female)</t>
+          <t>Trust in the court system</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.1793107796856119</v>
+        <v>0.2160488345528788</v>
       </c>
       <c r="E52" t="n">
-        <v>0.117996</v>
+        <v>0.0801529198470801</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+          <t>DIS Theme 7 - Political Vulnerability.csv</t>
         </is>
       </c>
     </row>
@@ -3896,14 +3896,14 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Female unemployment rate</t>
+          <t>Fear of movement or travel (female)</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.09927208999672819</v>
+        <v>0.1793107796856119</v>
       </c>
       <c r="E53" t="n">
-        <v>0.06526</v>
+        <v>0.117996</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -3932,14 +3932,14 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Reported incidents of gender-based violence</t>
+          <t>Female unemployment rate</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.1732225952812849</v>
+        <v>0.09927208999672819</v>
       </c>
       <c r="E54" t="n">
-        <v>0.114041</v>
+        <v>0.06526</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -3968,14 +3968,14 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Reports of harassment or violence</t>
+          <t>Reported incidents of gender-based violence</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.1726001793585464</v>
+        <v>0.1732225952812849</v>
       </c>
       <c r="E55" t="n">
-        <v>0.248517</v>
+        <v>0.114041</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -4004,14 +4004,14 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Safety at night (female)</t>
+          <t>Reports of harassment or violence</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.1902249072695776</v>
+        <v>0.1726001793585464</v>
       </c>
       <c r="E56" t="n">
-        <v>0.125247</v>
+        <v>0.248517</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -4040,14 +4040,14 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Service access difficulty (female)</t>
+          <t>Safety at night (female)</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.0924605433273403</v>
+        <v>0.1902249072695776</v>
       </c>
       <c r="E57" t="n">
-        <v>0.265656</v>
+        <v>0.125247</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -4076,26 +4076,62 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
+          <t>Service access difficulty (female)</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>0.0924605433273403</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.265656</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>8</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Gender Based Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
           <t>Trust in the court system</t>
         </is>
       </c>
-      <c r="D58" t="n">
+      <c r="D59" t="n">
         <v>0.0959478882479386</v>
       </c>
-      <c r="E58" t="n">
+      <c r="E59" t="n">
         <v>0.06328300000000001</v>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>custom</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
         <is>
           <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
         </is>

</xml_diff>

<commit_message>
Added Spider Web to Analysis Section
</commit_message>
<xml_diff>
--- a/Automated_Pipeline/CUSTOM/REPORTS/Indicator_Weights_Summary.xlsx
+++ b/Automated_Pipeline/CUSTOM/REPORTS/Indicator_Weights_Summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOV" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DIS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAD" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OVERALL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="GOV" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="DIS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CAD" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="OVERALL" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2084,7 +2084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.3033236464308781</v>
+        <v>0.3411693934857454</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3384084610576228</v>
+        <v>0.1442803396687116</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -3356,14 +3356,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Forest fire risk</t>
+          <t>Consecutive Dry Days</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.305085107923876</v>
+        <v>0.3244037381325479</v>
       </c>
       <c r="E38" t="n">
-        <v>0.3403736671339433</v>
+        <v>0.1371901536927267</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -3392,14 +3392,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Mean annual hot days</t>
+          <t>Consecutive Wet Days</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.287915307646844</v>
+        <v>0.3349491218135267</v>
       </c>
       <c r="E39" t="n">
-        <v>0.3212178718084338</v>
+        <v>0.1416497903672929</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -3419,27 +3419,27 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Political Vulnerability</t>
+          <t>Climate Change and Environmental Risk</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Demographic Factor</t>
+          <t>Days withh at least 10 mm rainfall</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.1310980037857101</v>
+        <v>0.2919332017636805</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>0.1234583825960877</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>kendall</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3449,33 +3449,33 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>DIS Theme 7 - Political Vulnerability.csv</t>
+          <t>DIS Theme 6 - Climate Change and Environmental Risk.csv</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Political Vulnerability</t>
+          <t>Climate Change and Environmental Risk</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Faith in elections</t>
+          <t>Days withh at least 20 mm rainfall</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.1591490072633531</v>
+        <v>0.2611856609596325</v>
       </c>
       <c r="E41" t="n">
-        <v>0.0549619450380549</v>
+        <v>0.1104552653297348</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>kendall</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3485,33 +3485,33 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>DIS Theme 7 - Political Vulnerability.csv</t>
+          <t>DIS Theme 6 - Climate Change and Environmental Risk.csv</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Political Vulnerability</t>
+          <t>Climate Change and Environmental Risk</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Faith in politics</t>
+          <t>Forest fire risk</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.165237380242456</v>
+        <v>0.2183581724823124</v>
       </c>
       <c r="E42" t="n">
-        <v>0.0427479572520427</v>
+        <v>0.092343545161836</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>kendall</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3521,33 +3521,33 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>DIS Theme 7 - Political Vulnerability.csv</t>
+          <t>DIS Theme 6 - Climate Change and Environmental Risk.csv</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Political Vulnerability</t>
+          <t>Climate Change and Environmental Risk</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ISF effect on quality of life: worsened life somewhat + alot</t>
+          <t>Hot days (Tmax &gt; 30°C)</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.2598686477891816</v>
+        <v>0.3358946682110201</v>
       </c>
       <c r="E43" t="n">
-        <v>0.0396949603050396</v>
+        <v>0.1420496613932634</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>kendall</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3557,33 +3557,33 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>DIS Theme 7 - Political Vulnerability.csv</t>
+          <t>DIS Theme 6 - Climate Change and Environmental Risk.csv</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Political Vulnerability</t>
+          <t>Climate Change and Environmental Risk</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LAF effect on quality of life: worsened life somewhat + alot</t>
+          <t>Very Hot Days (Tmax &gt; 35°C)</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.2432688551783794</v>
+        <v>0.256734476028247</v>
       </c>
       <c r="E44" t="n">
-        <v>0.0473279526720473</v>
+        <v>0.1085728617903465</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>kendall</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>DIS Theme 7 - Political Vulnerability.csv</t>
+          <t>DIS Theme 6 - Climate Change and Environmental Risk.csv</t>
         </is>
       </c>
     </row>
@@ -3608,14 +3608,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Municipal authorities effect on quality of life: worsened life somewhat + alot</t>
+          <t>Demographic Factor</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.1715002110059001</v>
+        <v>0.1310980037857101</v>
       </c>
       <c r="E45" t="n">
-        <v>0.0587789412210587</v>
+        <v>0</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -3644,14 +3644,14 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Municipal council entrenchment</t>
+          <t>Faith in elections</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.1136877556707401</v>
+        <v>0.1591490072633531</v>
       </c>
       <c r="E46" t="n">
-        <v>0.2267177732822267</v>
+        <v>0.0549619450380549</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -3680,14 +3680,14 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Municipal elections turnout</t>
+          <t>Faith in politics</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.1451036849467801</v>
+        <v>0.165237380242456</v>
       </c>
       <c r="E47" t="n">
-        <v>0.0519079480920519</v>
+        <v>0.0427479572520427</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -3716,14 +3716,14 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">State Citizen Incidents </t>
+          <t>ISF effect on quality of life: worsened life somewhat + alot</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.1034531739412614</v>
+        <v>0.2598686477891816</v>
       </c>
       <c r="E48" t="n">
-        <v>0.0358779641220358</v>
+        <v>0.0396949603050396</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -3752,14 +3752,14 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Trust in LAF</t>
+          <t>LAF effect on quality of life: worsened life somewhat + alot</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.1035566077800814</v>
+        <v>0.2432688551783794</v>
       </c>
       <c r="E49" t="n">
-        <v>0.0366409633590366</v>
+        <v>0.0473279526720473</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -3788,14 +3788,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Trust in Parliament</t>
+          <t>Municipal authorities effect on quality of life: worsened life somewhat + alot</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.210369020033815</v>
+        <v>0.1715002110059001</v>
       </c>
       <c r="E50" t="n">
-        <v>0.07786292213707779</v>
+        <v>0.0587789412210587</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -3824,14 +3824,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Trust in security forces</t>
+          <t>Municipal council entrenchment</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.2163576846840651</v>
+        <v>0.1136877556707401</v>
       </c>
       <c r="E51" t="n">
-        <v>0.2473277526722473</v>
+        <v>0.2267177732822267</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -3860,14 +3860,14 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Trust in the court system</t>
+          <t>Municipal elections turnout</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.2160488345528788</v>
+        <v>0.1451036849467801</v>
       </c>
       <c r="E52" t="n">
-        <v>0.0801529198470801</v>
+        <v>0.0519079480920519</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -3887,23 +3887,23 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Gender Based Vulnerabilities</t>
+          <t>Political Vulnerability</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Fear of movement or travel (female)</t>
+          <t xml:space="preserve">State Citizen Incidents </t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.1793107796856119</v>
+        <v>0.1034531739412614</v>
       </c>
       <c r="E53" t="n">
-        <v>0.117996</v>
+        <v>0.0358779641220358</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -3917,29 +3917,29 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+          <t>DIS Theme 7 - Political Vulnerability.csv</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Gender Based Vulnerabilities</t>
+          <t>Political Vulnerability</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Female unemployment rate</t>
+          <t>Trust in LAF</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.09927208999672819</v>
+        <v>0.1035566077800814</v>
       </c>
       <c r="E54" t="n">
-        <v>0.06526</v>
+        <v>0.0366409633590366</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -3953,29 +3953,29 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+          <t>DIS Theme 7 - Political Vulnerability.csv</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Gender Based Vulnerabilities</t>
+          <t>Political Vulnerability</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Reported incidents of gender-based violence</t>
+          <t>Trust in Parliament</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.1732225952812849</v>
+        <v>0.210369020033815</v>
       </c>
       <c r="E55" t="n">
-        <v>0.114041</v>
+        <v>0.07786292213707779</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -3989,29 +3989,29 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+          <t>DIS Theme 7 - Political Vulnerability.csv</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Gender Based Vulnerabilities</t>
+          <t>Political Vulnerability</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Reports of harassment or violence</t>
+          <t>Trust in security forces</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.1726001793585464</v>
+        <v>0.2163576846840651</v>
       </c>
       <c r="E56" t="n">
-        <v>0.248517</v>
+        <v>0.2473277526722473</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -4025,29 +4025,29 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+          <t>DIS Theme 7 - Political Vulnerability.csv</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Gender Based Vulnerabilities</t>
+          <t>Political Vulnerability</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Safety at night (female)</t>
+          <t>Trust in the court system</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.1902249072695776</v>
+        <v>0.2160488345528788</v>
       </c>
       <c r="E57" t="n">
-        <v>0.125247</v>
+        <v>0.0801529198470801</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+          <t>DIS Theme 7 - Political Vulnerability.csv</t>
         </is>
       </c>
     </row>
@@ -4076,14 +4076,14 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Service access difficulty (female)</t>
+          <t>Fear of movement or travel (female)</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.0924605433273403</v>
+        <v>0.1793107796856119</v>
       </c>
       <c r="E58" t="n">
-        <v>0.265656</v>
+        <v>0.117996</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -4112,26 +4112,206 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
+          <t>Female unemployment rate</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>0.09927208999672819</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.06526</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>8</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Gender Based Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Reported incidents of gender-based violence</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>0.1732225952812849</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.114041</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>8</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Gender Based Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Reports of harassment or violence</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>0.1726001793585464</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.248517</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>8</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Gender Based Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Safety at night (female)</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>0.1902249072695776</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.125247</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>8</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Gender Based Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Service access difficulty (female)</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0.0924605433273403</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.265656</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>8</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Gender Based Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
           <t>Trust in the court system</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D64" t="n">
         <v>0.0959478882479386</v>
       </c>
-      <c r="E59" t="n">
+      <c r="E64" t="n">
         <v>0.06328300000000001</v>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>custom</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
         <is>
           <t>DIS Theme 8 - Gender Based Vulnerabilities.csv</t>
         </is>
@@ -4148,7 +4328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4812,10 +4992,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.1007646363096458</v>
+        <v>0.1939943438925875</v>
       </c>
       <c r="E21" t="n">
-        <v>0.2775605518210395</v>
+        <v>0.1078682888424959</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -4844,14 +5024,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Forest fire risk</t>
+          <t>Consecutive Dry Days</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.0818067110770221</v>
+        <v>0.2598616094283791</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2253401262663915</v>
+        <v>0.1444930124376028</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -4880,14 +5060,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mean annual hot days</t>
+          <t>Consecutive Wet Days</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.1804652428223579</v>
+        <v>0.2648651664915811</v>
       </c>
       <c r="E23" t="n">
-        <v>0.4970993219125688</v>
+        <v>0.1472751818952455</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -4900,6 +5080,186 @@
         </is>
       </c>
       <c r="H23" t="inlineStr">
+        <is>
+          <t>CAD Theme 6 - Climate Change and Environmental Risk.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Climate Change and Environmental Risk</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Days withh at least 10 mm rainfall</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0.2914091934678101</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.1620346780303505</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>kendall</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>CAD Theme 6 - Climate Change and Environmental Risk.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Climate Change and Environmental Risk</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Days withh at least 20 mm rainfall</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>0.2182480739309751</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.1213542921186392</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>kendall</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>CAD Theme 6 - Climate Change and Environmental Risk.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Climate Change and Environmental Risk</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Forest fire risk</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0.1655909235332009</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0920748987365578</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>kendall</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>CAD Theme 6 - Climate Change and Environmental Risk.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Climate Change and Environmental Risk</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Hot days (Tmax &gt; 30°C)</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.1558228871577597</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0866434962119899</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>kendall</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>CAD Theme 6 - Climate Change and Environmental Risk.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>6</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Climate Change and Environmental Risk</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Very Hot Days (Tmax &gt; 35°C)</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0.2486450070843243</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.1382561517271182</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>kendall</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>CAD Theme 6 - Climate Change and Environmental Risk.csv</t>
         </is>
@@ -5192,10 +5552,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.2959183673469387</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1283185840707964</v>
+        <v>0.1166666666666666</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -5220,10 +5580,10 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.1326530612244897</v>
+        <v>0.1224489795918367</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0575221238938053</v>
+        <v>0.05</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -5248,10 +5608,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.4387755102040816</v>
+        <v>0.4081632653061224</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1902654867256637</v>
+        <v>0.1666666666666666</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -5276,10 +5636,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.3571428571428571</v>
+        <v>0.4081632653061224</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1548672566371681</v>
+        <v>0.1666666666666666</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -5304,10 +5664,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.3979591836734694</v>
+        <v>0.3877551020408162</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1725663716814159</v>
+        <v>0.1583333333333333</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -5332,10 +5692,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.2346938775510203</v>
+        <v>0.3061224489795918</v>
       </c>
       <c r="E15" t="n">
-        <v>0.1017699115044247</v>
+        <v>0.125</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -5360,10 +5720,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.2346938775510203</v>
+        <v>0.2653061224489795</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1017699115044247</v>
+        <v>0.1083333333333333</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -5388,10 +5748,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.2142857142857142</v>
+        <v>0.2653061224489795</v>
       </c>
       <c r="E17" t="n">
-        <v>0.09292035398230079</v>
+        <v>0.1083333333333333</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -5416,10 +5776,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.2254945054945055</v>
+        <v>0.2202197802197802</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1609159347553325</v>
+        <v>0.1510856453558504</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -5444,10 +5804,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.1481318681318681</v>
+        <v>0.1745054945054945</v>
       </c>
       <c r="E19" t="n">
-        <v>0.1057089084065244</v>
+        <v>0.1197225572979493</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -5472,10 +5832,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.1648351648351648</v>
+        <v>0.1903296703296703</v>
       </c>
       <c r="E20" t="n">
-        <v>0.1176286072772898</v>
+        <v>0.1305790108564535</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -5500,10 +5860,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.2536263736263737</v>
+        <v>0.243956043956044</v>
       </c>
       <c r="E21" t="n">
-        <v>0.18099121706399</v>
+        <v>0.1673703256936067</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -5528,10 +5888,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.2457142857142857</v>
+        <v>0.2386813186813186</v>
       </c>
       <c r="E22" t="n">
-        <v>0.17534504391468</v>
+        <v>0.163751507840772</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -5556,10 +5916,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.069010989010989</v>
+        <v>0.0971428571428571</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0492471769134253</v>
+        <v>0.06664656212303979</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -5584,10 +5944,10 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.1437362637362637</v>
+        <v>0.1375824175824176</v>
       </c>
       <c r="E24" t="n">
-        <v>0.1025721455457967</v>
+        <v>0.09439083232810611</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -5612,10 +5972,10 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.1507692307692307</v>
+        <v>0.1551648351648351</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1075909661229611</v>
+        <v>0.1064535585042219</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5640,10 +6000,10 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.0360288117909377</v>
+        <v>0.050720093460957</v>
       </c>
       <c r="E26" t="n">
-        <v>0.2565424071990172</v>
+        <v>0.1823730417167728</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5668,10 +6028,10 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.0484977771574825</v>
+        <v>0.066726416065733</v>
       </c>
       <c r="E27" t="n">
-        <v>0.3453274165125684</v>
+        <v>0.2399265977325954</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5696,10 +6056,10 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.0104094250547086</v>
+        <v>0.0122528591536715</v>
       </c>
       <c r="E28" t="n">
-        <v>0.07412009523346</v>
+        <v>0.0440573161660754</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5724,10 +6084,10 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.0212996846250575</v>
+        <v>0.0553722335478623</v>
       </c>
       <c r="E29" t="n">
-        <v>0.1516639626640862</v>
+        <v>0.1991006319132409</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -5752,10 +6112,10 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.0242042862628406</v>
+        <v>0.09304018986287819</v>
       </c>
       <c r="E30" t="n">
-        <v>0.172346118390868</v>
+        <v>0.3345424124713154</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>

</xml_diff>